<commit_message>
Stage: 장부방 8005 행 추가(Order 2), 8001→8005→8002 연결, Language 30027 추가 (10/30 김현호 확정)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CDH3mxXsBhjTgcPjfLvqYR
</commit_message>
<xml_diff>
--- a/tables/Stage.xlsx
+++ b/tables/Stage.xlsx
@@ -619,7 +619,7 @@
         <v>1</v>
       </c>
       <c r="E7" s="3" t="n">
-        <v>8002</v>
+        <v>8005</v>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
@@ -643,7 +643,7 @@
       </c>
       <c r="J7" s="3" t="inlineStr">
         <is>
-          <t>인트로 컷씬 뒤, 부상당한 피난민 NPC. 마을 안 장부방(결박 가르기 해금, 맵 2 전)</t>
+          <t>인트로 컷씬 뒤, 부상당한 피난민 NPC. 다음은 장부방(8005)</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
         <v>30012</v>
       </c>
       <c r="D8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E8" s="3" t="n">
         <v>8003</v>
@@ -699,7 +699,7 @@
         <v>30013</v>
       </c>
       <c r="D9" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E9" s="3" t="n">
         <v>8004</v>
@@ -739,7 +739,7 @@
         <v>30014</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
@@ -759,6 +759,42 @@
       <c r="J10" s="3" t="inlineStr">
         <is>
           <t>전투 BGM BPM 낮춤 버전(10/28)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>8005</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>장부방</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>30027</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" t="n">
+        <v>8002</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>BGM_VILLAGE</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="n"/>
+      <c r="H11" s="3" t="n"/>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>마을 안 작은 실내 맵. 몬스터 없음(스폰 파일 없음). 명부 조사(E) → 일러스트 연출로 결박 가르기 해금(10/30 확정)</t>
         </is>
       </c>
     </row>

</xml_diff>